<commit_message>
Fix all test cases - 35 tests now passing
</commit_message>
<xml_diff>
--- a/testdata/IT23210288.xlsx
+++ b/testdata/IT23210288.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\3rd year\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{057A1F5D-E5A4-49BE-A3E6-55B4E74D36C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A661509C-85B0-4441-97A7-CE4929EDCE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -118,12 +118,6 @@
     <t>Convert complex conditional sentence</t>
   </si>
   <si>
-    <t>oya enavaanam mama balan innavaa.</t>
-  </si>
-  <si>
-    <t>ඔයා එනවානම් මම බලන් ඉන්නවා.</t>
-  </si>
-  <si>
     <t>Complex conditional sentence structure is correctly handled.</t>
   </si>
   <si>
@@ -613,19 +607,7 @@
     <t>Missing 'a' in 'paan' (should be double vowel) causes incorrect Sinhala output 'පන්' instead of correct 'පාන්' (bread).</t>
   </si>
   <si>
-    <t>Copy button copies Sinhala output to clipboard</t>
-  </si>
-  <si>
-    <t>api paasal yanavaa</t>
-  </si>
-  <si>
-    <t>Clicking copy button should copy Sinhala output 'අපි පාසල් යනවා' to clipboard</t>
-  </si>
-  <si>
     <t>Pass</t>
-  </si>
-  <si>
-    <t>Copy button functionality works correctly. Sinhala text is copied to system clipboard and can be pasted into other applications without corruption.</t>
   </si>
   <si>
     <t>• Daily language usage
@@ -733,7 +715,25 @@
     <t>සුබ උදෑසනක්!</t>
   </si>
   <si>
-    <t>Pos_UI_0002</t>
+    <t>api yanavaanam apee ammaagen ahannam.</t>
+  </si>
+  <si>
+    <t>අපි යනවානම් අපේ අම්මාගෙන් අහන්නම්.</t>
+  </si>
+  <si>
+    <t>Pos_UI_0001</t>
+  </si>
+  <si>
+    <t>Verify real-time Sinhala output updates while typing</t>
+  </si>
+  <si>
+    <t>api kadeeta yanavaa.</t>
+  </si>
+  <si>
+    <t>Sinhala output updates in real-time while typing and displays: අපි කඩේට යනවා.</t>
+  </si>
+  <si>
+    <t>Real-time conversion works smoothly, with instant character-by-character updates, no noticeable lag, and a responsive UI.</t>
   </si>
 </sst>
 </file>
@@ -1198,13 +1198,13 @@
         <v>12</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>13</v>
@@ -1233,7 +1233,7 @@
         <v>18</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>19</v>
@@ -1253,16 +1253,16 @@
         <v>22</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>23</v>
@@ -1282,16 +1282,16 @@
         <v>22</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>27</v>
@@ -1311,193 +1311,193 @@
         <v>22</v>
       </c>
       <c r="D6" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="2" t="s">
+      <c r="F10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="E11" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="2" t="s">
+      <c r="F11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H11" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>59</v>
-      </c>
       <c r="I11" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="E12" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="2" t="s">
+      <c r="F12" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>14</v>
@@ -1505,231 +1505,231 @@
     </row>
     <row r="13" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="E13" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="E14" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="2" t="s">
+      <c r="I14" s="2" t="s">
         <v>73</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="E15" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2" t="s">
+      <c r="F15" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="E17" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="2" t="s">
+      <c r="F17" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H17" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="I17" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D18" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H18" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="I18" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="I18" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="E19" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>99</v>
-      </c>
       <c r="I19" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H20" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>14</v>
@@ -1737,28 +1737,28 @@
     </row>
     <row r="21" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="E21" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="F21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H21" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>109</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>14</v>
@@ -1766,437 +1766,437 @@
     </row>
     <row r="22" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H22" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>113</v>
-      </c>
-      <c r="F22" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="F23" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H23" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="I23" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="2" t="s">
+      <c r="F24" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H24" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E24" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="F24" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H24" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="I24" s="2" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="E25" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="2" t="s">
+      <c r="F25" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H25" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="I25" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="I25" s="2" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="E26" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="G26" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="2" t="s">
+      <c r="H26" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="G26" s="5" t="s">
+      <c r="I26" s="2" t="s">
         <v>136</v>
-      </c>
-      <c r="H26" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="85.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="F27" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H27" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B28" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="2" t="s">
+      <c r="F28" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="G28" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H28" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="I28" s="2" t="s">
         <v>146</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="F29" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H29" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="I29" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B30" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="2" t="s">
+      <c r="F30" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H30" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="I30" s="2" t="s">
         <v>154</v>
-      </c>
-      <c r="F30" s="2" t="s">
-        <v>194</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="I30" s="2" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="F31" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E31" s="2" t="s">
+      <c r="G31" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H31" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="F31" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H31" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="I31" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="79.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="2" t="s">
+      <c r="F32" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B33" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="2" t="s">
+      <c r="F33" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H33" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="I33" s="2" t="s">
         <v>168</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="I33" s="2" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="B34" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="2" t="s">
+      <c r="F34" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H34" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="E34" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="F34" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="G34" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H34" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="I34" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B35" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="H35" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="G35" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>177</v>
-      </c>
       <c r="I35" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="H36" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="F36" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="H36" s="2" t="s">
-        <v>182</v>
-      </c>
       <c r="I36" s="2" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="64.95" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>